<commit_message>
Meu progresso na UC6
</commit_message>
<xml_diff>
--- a/UC06_Aula12.xlsx
+++ b/UC06_Aula12.xlsx
@@ -413,39 +413,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>nome</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>idade</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>altura</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>ui</t>
-        </is>
+      <c r="A2" t="n">
+        <v>0</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>7</v>
+          <t>ANa</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>('75',)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>(1.78,)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>